<commit_message>
generate excel with comments and datetype from db query works
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -425,18 +425,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>column_name</t>
+          <t>Column Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>data_type</t>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
         </is>
       </c>
     </row>
@@ -451,6 +456,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -463,6 +469,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -475,6 +482,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -487,6 +495,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -499,6 +508,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -508,7 +518,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>double precision</t>
+          <t>float8</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The geographical origin of the sample as defined by latitude. The values should be reported in decimal degrees as precise as possible (max. 8 decimal points).</t>
         </is>
       </c>
     </row>
@@ -520,9 +535,10 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>double precision</t>
-        </is>
-      </c>
+          <t>float8</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -535,6 +551,7 @@
           <t>date</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -547,6 +564,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -559,6 +577,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -571,6 +590,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -583,6 +603,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -592,9 +613,10 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>double precision</t>
-        </is>
-      </c>
+          <t>float8</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -607,6 +629,7 @@
           <t>int4range</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -619,6 +642,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -628,9 +652,10 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>double precision</t>
-        </is>
-      </c>
+          <t>float8</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -640,9 +665,10 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>double precision</t>
-        </is>
-      </c>
+          <t>float8</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -655,6 +681,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -667,6 +694,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -679,6 +707,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -691,6 +720,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -703,6 +733,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -715,6 +746,7 @@
           <t>int4range</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -724,9 +756,10 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>double precision</t>
-        </is>
-      </c>
+          <t>float8</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -739,6 +772,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -751,6 +785,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -763,6 +798,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -775,6 +811,7 @@
           <t>date</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -787,6 +824,7 @@
           <t>date</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -799,6 +837,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -811,6 +850,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -823,6 +863,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -835,6 +876,7 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -847,11 +889,12 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>database_insert_by</t>
+          <t>Data inserter</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -859,11 +902,12 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>from_spreadsheet</t>
+          <t xml:space="preserve">External sample provider(s) email </t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -871,54 +915,20 @@
           <t>text</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>database_insert_datetime_utc</t>
+          <t>Full name of external sample provider(s)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>timestamp with time zone</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Data inserter</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">External sample provider(s) email </t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Full name of external sample provider(s)</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>